<commit_message>
Debug attendance flow and fix minor issues
</commit_message>
<xml_diff>
--- a/uploads/1781009236664-attendance.xlsx
+++ b/uploads/1781009236664-attendance.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:K61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,9 @@
       <c r="J1" t="str">
         <v>09 Jun 2026</v>
       </c>
+      <c r="K1" t="str">
+        <v>18 Jun 2026</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -462,6 +465,9 @@
       <c r="J2" t="str">
         <v/>
       </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -494,6 +500,9 @@
       <c r="J3" t="str">
         <v/>
       </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -526,6 +535,9 @@
       <c r="J4" t="str">
         <v/>
       </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -558,6 +570,9 @@
       <c r="J5" t="str">
         <v/>
       </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -590,6 +605,9 @@
       <c r="J6" t="str">
         <v/>
       </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -622,6 +640,9 @@
       <c r="J7" t="str">
         <v/>
       </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -654,6 +675,9 @@
       <c r="J8" t="str">
         <v/>
       </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -686,6 +710,9 @@
       <c r="J9" t="str">
         <v/>
       </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -718,6 +745,9 @@
       <c r="J10" t="str">
         <v/>
       </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -750,6 +780,9 @@
       <c r="J11" t="str">
         <v/>
       </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -782,6 +815,9 @@
       <c r="J12" t="str">
         <v/>
       </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -814,6 +850,9 @@
       <c r="J13" t="str">
         <v/>
       </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -846,6 +885,9 @@
       <c r="J14" t="str">
         <v/>
       </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -878,6 +920,9 @@
       <c r="J15" t="str">
         <v/>
       </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -910,6 +955,9 @@
       <c r="J16" t="str">
         <v/>
       </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -942,6 +990,9 @@
       <c r="J17" t="str">
         <v/>
       </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -974,6 +1025,9 @@
       <c r="J18" t="str">
         <v/>
       </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -1006,6 +1060,9 @@
       <c r="J19" t="str">
         <v/>
       </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -1038,6 +1095,9 @@
       <c r="J20" t="str">
         <v/>
       </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -1070,6 +1130,9 @@
       <c r="J21" t="str">
         <v/>
       </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -1102,6 +1165,9 @@
       <c r="J22" t="str">
         <v/>
       </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -1134,6 +1200,9 @@
       <c r="J23" t="str">
         <v/>
       </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -1166,6 +1235,9 @@
       <c r="J24" t="str">
         <v/>
       </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -1198,6 +1270,9 @@
       <c r="J25" t="str">
         <v/>
       </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -1230,6 +1305,9 @@
       <c r="J26" t="str">
         <v/>
       </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -1262,6 +1340,9 @@
       <c r="J27" t="str">
         <v/>
       </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -1294,6 +1375,9 @@
       <c r="J28" t="str">
         <v/>
       </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -1326,6 +1410,9 @@
       <c r="J29" t="str">
         <v/>
       </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -1358,6 +1445,9 @@
       <c r="J30" t="str">
         <v/>
       </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -1390,6 +1480,9 @@
       <c r="J31" t="str">
         <v/>
       </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -1422,6 +1515,9 @@
       <c r="J32" t="str">
         <v/>
       </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -1454,6 +1550,9 @@
       <c r="J33" t="str">
         <v/>
       </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -1486,6 +1585,9 @@
       <c r="J34" t="str">
         <v/>
       </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -1518,6 +1620,9 @@
       <c r="J35" t="str">
         <v/>
       </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -1550,6 +1655,9 @@
       <c r="J36" t="str">
         <v/>
       </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -1582,6 +1690,9 @@
       <c r="J37" t="str">
         <v/>
       </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -1614,6 +1725,9 @@
       <c r="J38" t="str">
         <v/>
       </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -1646,6 +1760,9 @@
       <c r="J39" t="str">
         <v/>
       </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -1678,6 +1795,9 @@
       <c r="J40" t="str">
         <v/>
       </c>
+      <c r="K40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -1710,6 +1830,9 @@
       <c r="J41" t="str">
         <v/>
       </c>
+      <c r="K41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -1742,6 +1865,9 @@
       <c r="J42" t="str">
         <v/>
       </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -1774,6 +1900,9 @@
       <c r="J43" t="str">
         <v/>
       </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -1806,6 +1935,9 @@
       <c r="J44" t="str">
         <v/>
       </c>
+      <c r="K44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -1838,6 +1970,9 @@
       <c r="J45" t="str">
         <v/>
       </c>
+      <c r="K45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -1870,6 +2005,9 @@
       <c r="J46" t="str">
         <v/>
       </c>
+      <c r="K46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -1902,6 +2040,9 @@
       <c r="J47" t="str">
         <v/>
       </c>
+      <c r="K47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -1934,6 +2075,9 @@
       <c r="J48" t="str">
         <v/>
       </c>
+      <c r="K48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -1966,6 +2110,9 @@
       <c r="J49" t="str">
         <v/>
       </c>
+      <c r="K49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -1998,6 +2145,9 @@
       <c r="J50" t="str">
         <v/>
       </c>
+      <c r="K50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -2030,6 +2180,9 @@
       <c r="J51" t="str">
         <v/>
       </c>
+      <c r="K51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -2062,6 +2215,9 @@
       <c r="J52" t="str">
         <v/>
       </c>
+      <c r="K52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -2094,6 +2250,9 @@
       <c r="J53" t="str">
         <v/>
       </c>
+      <c r="K53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -2126,6 +2285,9 @@
       <c r="J54" t="str">
         <v/>
       </c>
+      <c r="K54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -2158,6 +2320,9 @@
       <c r="J55" t="str">
         <v/>
       </c>
+      <c r="K55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -2190,6 +2355,9 @@
       <c r="J56" t="str">
         <v/>
       </c>
+      <c r="K56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -2222,6 +2390,9 @@
       <c r="J57" t="str">
         <v>P</v>
       </c>
+      <c r="K57" t="str">
+        <v>P</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -2254,6 +2425,9 @@
       <c r="J58" t="str">
         <v/>
       </c>
+      <c r="K58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -2286,6 +2460,9 @@
       <c r="J59" t="str">
         <v/>
       </c>
+      <c r="K59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -2318,6 +2495,9 @@
       <c r="J60" t="str">
         <v/>
       </c>
+      <c r="K60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -2350,10 +2530,13 @@
       <c r="J61" t="str">
         <v/>
       </c>
+      <c r="K61" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>